<commit_message>
feat(isotope): full MRM/MS1 isotopic interference correction
Two-level derive_interferences(): fragment-based MRM front/back overlaps via
ported LICAR class chemistry, and native MS1 whole-molecule M+2. Both feed the
extended correct_interferences() engine. Adds the mrm_pattern feature-metadata
input with import validation, the openxlsx2 template dropdown generator + round
-trip drift guard, and the manual reference article + tutorial rewrite.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/mrmhub_metadata_templates.xlsx
+++ b/inst/extdata/mrmhub_metadata_templates.xlsx
@@ -13,14 +13,21 @@
     <workbookView xWindow="13060" yWindow="3140" windowWidth="22940" windowHeight="19140" xr2:uid="{7A04E2C8-868F-5640-98CB-88D372530A12}"/>
   </bookViews>
   <sheets>
-    <sheet name="Info" sheetId="6" r:id="rId1"/>
-    <sheet name="Analyses" sheetId="1" r:id="rId2"/>
-    <sheet name="Features" sheetId="2" r:id="rId3"/>
-    <sheet name="ISTDs" sheetId="3" r:id="rId4"/>
-    <sheet name="ResponseCurves" sheetId="4" r:id="rId5"/>
-    <sheet name="QCconcentrations" sheetId="5" r:id="rId6"/>
+    <sheet name="Info" sheetId="6" state="visible" r:id="rId1"/>
+    <sheet name="Analyses" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Features" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="ISTDs" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="ResponseCurves" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="QCconcentrations" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="lists" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames>
+    <definedName name="AllPatterns">'lists'!$A$2:$A$60</definedName>
+    <definedName name="AllPatternsPos">'lists'!$B$2:$B$32</definedName>
+    <definedName name="AllPatternsNeg">'lists'!$C$2:$C$30</definedName>
+    <definedName name="polarities">'lists'!$D$2:$D$3</definedName>
+    <definedName name="prefix_map">'lists'!$E$2:$F$60</definedName>
+  </definedNames>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,12 +45,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" mc:Ignorable="xr">
   <authors>
     <author>Bo Burla</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{4389BCD8-3F95-1C46-9EA2-B891D9146321}">
+    <comment ref="A1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -76,7 +83,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{131224DE-51A7-264D-890E-DDBEE855070E}">
+    <comment ref="B1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -444,7 +451,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{EDC928AC-504D-5748-8AC2-B1928EDAEB8B}">
+    <comment ref="C1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -468,7 +475,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{33DD803C-E8D6-BE40-9EBA-C5C7C36AEDF0}">
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -501,7 +508,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{E5D987A4-9E6F-974C-AFF2-71E66A719782}">
+    <comment ref="E1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -535,7 +542,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{57E8468A-A3F7-6A48-BF6B-4A50A4032BE3}">
+    <comment ref="F1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -569,7 +576,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{ECB71D09-F433-9C40-A92D-C4F0DA18626E}">
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -612,7 +619,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{7FFEA4B3-C3E8-4C4E-8AB9-DF1C2CEC59CC}">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -651,12 +658,13 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" mc:Ignorable="xr">
   <authors>
     <author>Bo Burla</author>
+    <author>mrmhub</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{16FE6C21-CA03-1441-BD72-CF012FC68DCE}">
+    <comment ref="A1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -669,7 +677,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{DB5433A8-F188-7940-A3C8-6BDA1F2604F0}">
+    <comment ref="B1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -682,7 +690,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{27442A7B-33A5-4948-9D41-F3AD72F7D7EE}">
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -706,7 +714,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{297E3E24-8E52-E643-86C3-FE542885F038}">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -721,7 +729,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{BFB73AF3-8C54-FD4D-8D50-B4D016BF17E4}">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -735,7 +743,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{FF45CEA9-B8B0-B440-A6C2-124FD3ECBC64}">
+    <comment ref="K1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -749,7 +757,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{73925DE5-C144-0445-BE9E-63FF775D2D45}">
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -760,6 +768,52 @@
           </rPr>
           <t>Optional
 Positive value typically between 0 and 1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">mrmhub:</t>
+        </r>
+        <r>
+          <rPr/>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr/>
+          <t xml:space="preserve">polarity (optional): Pos or Neg. If set, it narrows the mrm_pattern choices. Leave blank to see all patterns.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="1">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">mrmhub:</t>
+        </r>
+        <r>
+          <rPr/>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr/>
+          <t xml:space="preserve">mrm_pattern: the class + MRM pattern for this feature, used by derive_interferences(). Pick from the dropdown; choices narrow with polarity if set. A name/pattern class mismatch is highlighted and warned about on import.</t>
         </r>
       </text>
     </comment>
@@ -768,12 +822,12 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" mc:Ignorable="xr">
   <authors>
     <author>Bo Burla</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{39CD8FB1-BAB4-5342-8523-663CDDCC094A}">
+    <comment ref="A1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -786,7 +840,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{A41AE4CE-AE3D-0B4C-84D1-2A73E3649821}">
+    <comment ref="B1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -800,7 +854,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{774B5792-4D0A-424F-8698-961764A4C201}">
+    <comment ref="C1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -819,12 +873,12 @@
 </file>
 
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" mc:Ignorable="xr">
   <authors>
     <author>Bo Burla</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{129C2C42-EB69-0547-A11C-306E3D0873D9}">
+    <comment ref="A1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -837,7 +891,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{3537029F-3C57-4A4C-9344-11D07937FF40}">
+    <comment ref="B1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -850,7 +904,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{83F02A22-8D9C-2C44-9D89-96E7FC818BFD}">
+    <comment ref="C1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -868,12 +922,12 @@
 </file>
 
 <file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" mc:Ignorable="xr">
   <authors>
     <author>Bo Burla</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{E73C7646-8E9A-224B-9A68-E2BE720D7EF6}">
+    <comment ref="A1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -886,7 +940,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{8295C253-AD69-DC43-A4A2-80A14178990A}">
+    <comment ref="B1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -909,7 +963,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{FA8C09F3-CA75-2A43-8A1D-703D322E3D87}">
+    <comment ref="C1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -922,7 +976,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{14BC61A4-4873-8F42-B3D1-93092B22F15D}">
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -935,7 +989,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{608C44CB-EA0C-1944-8482-E7A9EEA64394}">
+    <comment ref="E1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -953,7 +1007,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t>analysis_id</t>
   </si>
@@ -1185,8 +1239,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="37" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="37">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1911,7 +1965,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1964,8 +2018,27 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFEB3B"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
       <color rgb="FFF2F2F2"/>
@@ -2375,7 +2448,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{961DD4A9-4670-5445-B9CF-918B68BB1A53}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
@@ -2388,12 +2461,12 @@
     <col min="4" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="3" ht="30" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="3" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" s="3" ht="13" customFormat="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
     </row>
     <row r="3" spans="1:3" s="19" customFormat="1" x14ac:dyDescent="0.2">
@@ -2476,12 +2549,12 @@
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:4" s="8" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" s="8" ht="22" customFormat="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:4" s="8" customFormat="1" ht="10" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" s="8" ht="10" customFormat="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="7"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -2670,7 +2743,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F1A2D03-4C83-7448-999B-AC6C8C01C8BE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <tabColor theme="3" tint="0.749992370372631"/>
   </sheetPr>
@@ -2717,73 +2790,132 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA4946AB-D291-A441-8BD4-AFE744BDE9E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="34.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" bestFit="1" customWidth="1" width="34.83203125"/>
+    <col min="3" max="3" customWidth="1" width="14"/>
+    <col min="4" max="6" customWidth="1" width="12"/>
+    <col min="7" max="7" bestFit="1" customWidth="1" width="11.83203125"/>
+    <col min="8" max="8" bestFit="1" customWidth="1" width="14.1640625"/>
+    <col min="10" max="10" bestFit="1" customWidth="1" width="14.6640625"/>
+    <col min="11" max="11" bestFit="1" customWidth="1" hidden="false" width="9.625"/>
+    <col min="12" max="12" bestFit="1" customWidth="1" hidden="false" width="26.625"/>
+    <col min="13" max="13" bestFit="1" customWidth="1" width="7.6640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="F1" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="J1" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="21" t="s">
-        <v>14</v>
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>feature_id</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>istd_feature_id</t>
+        </is>
+      </c>
+      <c r="C1" s="21" t="inlineStr">
+        <is>
+          <t>feature_class</t>
+        </is>
+      </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>analyte_id</t>
+        </is>
+      </c>
+      <c r="E1" s="21" t="inlineStr">
+        <is>
+          <t>chem_formula</t>
+        </is>
+      </c>
+      <c r="F1" s="21" t="inlineStr">
+        <is>
+          <t>molecular_weight</t>
+        </is>
+      </c>
+      <c r="G1" s="21" t="inlineStr">
+        <is>
+          <t>feature_label</t>
+        </is>
+      </c>
+      <c r="H1" s="21" t="inlineStr">
+        <is>
+          <t>response_factor</t>
+        </is>
+      </c>
+      <c r="I1" s="21" t="inlineStr">
+        <is>
+          <t>is_quantifier</t>
+        </is>
+      </c>
+      <c r="J1" s="21" t="inlineStr">
+        <is>
+          <t>valid_integration</t>
+        </is>
+      </c>
+      <c r="K1" s="21" t="inlineStr">
+        <is>
+          <t>polarity</t>
+        </is>
+      </c>
+      <c r="L1" s="21" t="inlineStr">
+        <is>
+          <t>mrm_pattern</t>
+        </is>
+      </c>
+      <c r="M1" s="21" t="inlineStr">
+        <is>
+          <t>interference_feature_id</t>
+        </is>
+      </c>
+      <c r="N1" s="21" t="inlineStr">
+        <is>
+          <t>interference_proportion</t>
+        </is>
+      </c>
+      <c r="O1" s="21" t="inlineStr">
+        <is>
+          <t>remarks</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="K2:L501">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>AND($K2&lt;&gt;"",$L2&lt;&gt;"",ISNA(MATCH($L2,INDIRECT("AllPatterns"&amp;$K2),0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A501">
+    <cfRule type="expression" dxfId="6" priority="2">
+      <formula>AND($A2&lt;&gt;"",$L2&lt;&gt;"",NOT(ISNA(MATCH($L2,INDIRECT("AllPatterns"&amp;$K2),0))),LEFT($A2,LEN(VLOOKUP($L2,prefix_map,2,FALSE))+1)&lt;&gt;(VLOOKUP($L2,prefix_map,2,FALSE)&amp;" "))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L501">
+    <cfRule type="expression" dxfId="6" priority="3">
+      <formula>AND($A2&lt;&gt;"",$L2&lt;&gt;"",NOT(ISNA(MATCH($L2,INDIRECT("AllPatterns"&amp;$K2),0))),LEFT($A2,LEN(VLOOKUP($L2,prefix_map,2,FALSE))+1)&lt;&gt;(VLOOKUP($L2,prefix_map,2,FALSE)&amp;" "))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K501" errorStyle="stop">
+      <formula1>polarities</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L501" errorStyle="stop">
+      <formula1>INDIRECT("AllPatterns"&amp;$K2)</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CEF20C9-E726-8549-8B20-6F3F3BE0DDC1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
@@ -2812,7 +2944,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CE58D19-DFF1-D346-8279-6C7641F36845}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <tabColor theme="0" tint="-0.14999847407452621"/>
   </sheetPr>
@@ -2845,7 +2977,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17873042-8AD3-9A48-A30C-3D8A9EB1C366}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
@@ -2880,4 +3012,1361 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:F60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AllPatterns</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>AllPatternsPos</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>AllPatternsNeg</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>polarities</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>prefix</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AcylCarnitine (Pos) Pro=85</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AcylCarnitine (Pos) Pro=85</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>LPC d9 Pro=193.1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Pos</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AcylCarnitine (Pos) Pro=85</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>AcylCarnitine</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LPC (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LPC (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LPE (Neg) Pro=196.1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Neg</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>LPC (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>LPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LPC (Pos) Pro=104.1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LPC (Pos) Pro=104.1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PE (Neg) Pro=196.1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>LPC (Pos) Pro=104.1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>LPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LPC d9 Pro=193.1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LPC d9 Pro=193.1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PG (Neg) Pro=153</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>LPC d9 Pro=193.1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>LPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LPC-O (Pos) Pro=104.1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LPC-O (Pos) Pro=104.1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PI (Neg) Pro=241</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LPC-O (Pos) Pro=104.1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>LPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LPC-O (Pos, qualifier) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LPC-O (Pos, qualifier) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PS (Neg) Pre-Pro=87</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LPC-O (Pos, qualifier) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>LPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LPE (Pos) Pre-Pro=141</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LPE (Pos) Pre-Pro=141</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CL (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LPE (Pos) Pre-Pro=141</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>LPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LPE (Neg) Pro=196.1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LPI (Pos) Pre-Pro=277</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>LPC (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LPE (Neg) Pro=196.1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>LPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LPI (Pos) Pre-Pro=277</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PC (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>LPC (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LPI (Pos) Pre-Pro=277</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>LPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PC (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PCO (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>LPC (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PC (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PCO (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PCP (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LPE (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PCO (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PCP (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PE (Pos) Pre-Pro=141</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>LPI (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PCP (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PE (Pos) Pre-Pro=141</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PG (Pos) Pre-Pro=189</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LPG (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PE (Pos) Pre-Pro=141</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PE (Neg) Pro=196.1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PI (Pos) Pre-Pro=277</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FA (Neg) SIM</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PE (Neg) Pro=196.1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PG (Pos) Pre-Pro=189</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PS (Pos) Pre-Pro=185</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PC (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PG (Pos) Pre-Pro=189</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PG (Neg) Pro=153</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>S1P (Pos) Pro=60.1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PCO (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PG (Neg) Pro=153</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PI (Pos) Pre-Pro=277</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>S1Pql (Pos, QL) Pro=113</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PCP (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PI (Pos) Pre-Pro=277</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PI (Neg) Pro=241</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SM (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PC (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PI (Neg) Pro=241</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PS (Pos) Pre-Pro=185</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PE-P (Pos) FA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PC (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>PS (Pos) Pre-Pro=185</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PS (Neg) Pre-Pro=87</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hex1Sph (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PCO (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PS (Neg) Pre-Pro=87</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S1P (Pos) Pro=60.1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>PCO (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>S1P (Pos) Pro=60.1</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>S1P</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S1Pql (Pos, QL) Pro=113</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>deoxyCer (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PCP (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>S1Pql (Pos, QL) Pro=113</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>S1P</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SM (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>dhCer (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PCP (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SM (Pos) Pro=184.1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CL (Neg) FA</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>dhCer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PE (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CL (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>LPC (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GM3 (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PEO (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LPC (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>LPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LPC (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Hex1Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PEP (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LPC (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>LPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LPC (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Hex2Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PG (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LPC (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>LPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LPE (Neg) FA</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Hex3Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PI (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LPE (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>LPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LPI (Neg) FA</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CE (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>PS (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LPI (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>LPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LPG (Neg) FA</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DG (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LPG (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>LPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FA (Neg) SIM</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TG (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>FA (Neg) SIM</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PC (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>PC (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PCO (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PCO (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PCP (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>PCP (Neg, FA) FA</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PC (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>PC (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PC (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>PC (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PCO (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PCO (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PCO (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>PCO (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PCP (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PCP (Neg, AA) FA</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PCP (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>PCP (Neg, -CH3) FA</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PE (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>PE (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PEO (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PEO (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PEP (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PEP (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PE-P (Pos) FA</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>PE-P (Pos) FA</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PG (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>PG (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PI (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>PI (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PS (Neg) FA</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>PS (Neg) FA</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Hex1Sph (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Hex1Sph (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Hex1Sph</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Cer</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>deoxyCer (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>deoxyCer (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>deoxyCer</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>dhCer (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>dhCer (Pos) SphB-H2O</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>dhCer</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>dhCer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>dhCer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>dhCer</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>GM3 (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>GM3 (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>GM3</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Hex1Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Hex1Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Hex1Cer</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Hex2Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Hex2Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Hex2Cer</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Hex3Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Hex3Cer (Pos) SphB-2H2O</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Hex3Cer</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CE (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>CE (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>DG (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>DG (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>TG (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TG (Pos) FANL</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TG</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>